<commit_message>
fix: corrige bordas ausentes nas celulas RNF58 e RF62 da planilha de feedbacks
As celulas de Decisao da equipe e Justificativa preenchidas no commit
anterior (RNF58 e RF62) nao tinham nenhum estilo de borda no arquivo
original, diferente do resto da tabela. Copia a borda das celulas
vizinhas da mesma linha e regera o PDF.
</commit_message>
<xml_diff>
--- a/docs/assets/Feedbacks_semrequisitos_to_storm_com_decisoes.xlsx
+++ b/docs/assets/Feedbacks_semrequisitos_to_storm_com_decisoes.xlsx
@@ -74,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -100,6 +100,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2727,12 +2730,12 @@
           <t>Nenhum ajuste necessário.</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="10" t="inlineStr">
         <is>
           <t>Não aplicável</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G63" s="10" t="inlineStr">
         <is>
           <t>Nenhum problema identificado.</t>
         </is>
@@ -11512,12 +11515,12 @@
           <t>Manter apenas a extensão responsiva até 1920 pixels.</t>
         </is>
       </c>
-      <c r="F59" s="0" t="inlineStr">
+      <c r="F59" s="10" t="inlineStr">
         <is>
           <t>Aceito</t>
         </is>
       </c>
-      <c r="G59" s="0" t="inlineStr">
+      <c r="G59" s="10" t="inlineStr">
         <is>
           <t>O refluxo em 320 pixels foi reconhecido como parte do RNF56 (critério 1.4.10), e o RNF58 passou a tratar apenas da extensão responsiva até 1920 pixels, com as larguras de verificação definidas.</t>
         </is>

</xml_diff>